<commit_message>
Remove redundant void level
</commit_message>
<xml_diff>
--- a/LangMod/EN/SourcePod.xlsx
+++ b/LangMod/EN/SourcePod.xlsx
@@ -695,7 +695,7 @@
   <dimension ref="A1:XFD5"/>
   <sheetFormatPr defaultColWidth="7.5078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="6.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="29.12"/>
@@ -711,7 +711,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="7.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="3" width="5.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="6.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="2.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="10.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="8.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="6.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="42.29"/>
@@ -1127,7 +1127,7 @@
     <row r="3" s="10" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="n">
-        <f aca="false">MAX(B4:B9965)</f>
+        <f aca="false">MAX(B4:B9951)</f>
         <v>42000</v>
       </c>
       <c r="C3" s="5"/>

</xml_diff>